<commit_message>
Clean up dynamic duplicates, fix RAN capacity attribution to TelTech/Comclark, and reconcile master comparison
</commit_message>
<xml_diff>
--- a/FWA_Metric_to_Source_Mapping.xlsx
+++ b/FWA_Metric_to_Source_Mapping.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Metric to Source Mapping" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Source Datasets &amp; Repositories" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Regulatory &amp; Engineering Stds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric to Source Mapping" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Datasets &amp; Repositories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regulatory &amp; Engineering Stds" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -529,7 +529,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -553,6 +553,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1053,7 +1054,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>3GPP / TelTech RAN Engineering</t>
+          <t>TelTech &amp; Comclark RAN Engineering (Referencing 3GPP TS 38.104)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -1064,7 +1065,7 @@
       <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Modeled: = ROUNDUP(Target Subs @ 30% / 1,000, 0)
-Dimensioned strictly for 1,000 subscribers per BTS total across 3 sectors (~333 subs/sector).</t>
+Dimensioned for 1,000 subscribers per BTS total across 3 sectors (~333 subs/sector). Note: 3GPP TS 38.104 defines Band n50 RF specifications and 100MHz bandwidth, while the 1,000 subs/node capacity target is TelTech &amp; Comclark's RAN capacity planning standard.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1223,7 +1224,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
@@ -1462,7 +1463,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>

</xml_diff>